<commit_message>
feat(rop): implement Re-order Paragraph practice mode and clean up RMCMA accessibility and keys
</commit_message>
<xml_diff>
--- a/public/database/RMCMA/RMCMA/RMCMA.xlsx
+++ b/public/database/RMCMA/RMCMA/RMCMA.xlsx
@@ -1713,53 +1713,21 @@
 ---
 [] explain Edison's financial success
 [x] describe the model used to design Kinetoscope parlors
-[x] contrast their operational modes and commercial focuses with those of Kinetoscope parlors
+[] contrast their operational modes and commercial focuses with those of Kinetoscope parlors
 [] illustrate how much more technologically advanced Kinetoscope parlors were
 [] emphasize that phonograph parlors were more profitable than Kinetoscope parlors</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Understanding the author's purpose is a key skill in PTE Academic, and we'll analyze each option carefully to see how it aligns with the passage.&lt;/p&gt;
-&lt;p&gt;Here's a detailed analysis:&lt;/p&gt;
-&lt;h3&gt;Passage Analysis:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;The passage introduces Kinetoscope arcades and immediately links them to phonograph parlors, stating they were "modeled on" them.&lt;/li&gt;
-    &lt;li&gt;It describes the operation of phonograph parlors: individual listening through ear tubes, moving from machine to machine.&lt;/li&gt;
-    &lt;li&gt;It then explicitly states Kinetoscope parlors "functioned in a similar way."&lt;/li&gt;
-    &lt;li&gt;The passage then shifts focus to Edison's commercial strategy for Kinetoscopes: he was more interested in selling expensive machines ($1,000 each) than the cheaper films ($10-$15 each).&lt;/li&gt;
-    &lt;li&gt;Crucially, Edison refused to develop projection technology because he wanted exhibitors to buy *multiple* Kinetoscopes instead of just *one* projector.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Question Analysis:&lt;/h3&gt;
-&lt;p&gt;The question asks for the author's purpose in discussing phonograph parlors. This means we need to identify *why* the author brought them up in the context of Kinetoscopes.&lt;/p&gt;
-&lt;h3&gt;Option Analysis:&lt;/h3&gt;
-&lt;h4&gt;Correct Options:&lt;/h4&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;strong&gt;describe the model used to design Kinetoscope parlors&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is strongly supported by the very first sentence of the passage: "These Kinetoscope arcades were &lt;strong&gt;modeled on phonograph parlors&lt;/strong&gt;..." The passage then describes how phonograph parlors operated ("customers listened to recordings through individual ear tubes, moving from one machine to the next") and immediately follows with, "The Kinetoscope parlors &lt;strong&gt;functioned in a similar way&lt;/strong&gt;." This clearly indicates that phonograph parlors served as the blueprint or design model for Kinetoscope parlors. The author discusses them to establish this foundational similarity.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;strong&gt;contrast their operational modes and commercial focuses with those of Kinetoscope parlors&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option requires a more nuanced understanding. While the passage explicitly states that Kinetoscope parlors "functioned in a similar way" (suggesting similarity in operational mode, not contrast), the discussion of phonograph parlors sets the stage for a contrast in *commercial focus*. The phonograph parlors are mentioned as having "proven successful," but their specific commercial strategy isn't detailed. In contrast, the passage then elaborates extensively on Edison's very specific and calculated *commercial focus* for Kinetoscopes: selling expensive machines ($1,000 apiece) and deliberately refusing to develop projection technology to ensure multiple sales. This detailed, machine-centric commercial strategy for Kinetoscopes is presented as a distinct approach compared to the general "success" of phonograph parlors. Therefore, the author uses the phonograph parlors as a point of reference to highlight the unique and deliberate commercial decisions Edison made for the Kinetoscope business, thereby contrasting the *nature* and *specificity* of the commercial focuses discussed for each.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;h4&gt;Incorrect Options:&lt;/h4&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;strong&gt;explain Edison's financial success&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; While the passage mentions that phonograph parlors "had proven successful for Edison several years earlier," the primary purpose of discussing them isn't to *explain* the details of that success. It's a brief statement of fact used as background to introduce the Kinetoscope parlors. The passage doesn't delve into *how* or *why* they were financially successful; it merely states that they were. The focus quickly shifts to Edison's strategy for Kinetoscopes.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;strong&gt;illustrate how much more technologically advanced Kinetoscope parlors were&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage does not suggest that Kinetoscope parlors were technologically *more advanced* than phonograph parlors. In fact, it emphasizes their *similarity* in function: "The Kinetoscope parlors functioned in a similar way." The difference was in the medium (visual vs. audio), not necessarily a leap in the underlying technology of the parlor model itself.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;strong&gt;emphasize that phonograph parlors were more profitable than Kinetoscope parlors&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage states phonograph parlors were "successful," but it never makes a direct comparison of profitability between phonograph and Kinetoscope parlors. It discusses Edison's *interest* in selling Kinetoscopes for a high price, implying potential profitability for him, but it doesn't state that one type of parlor was more profitable than the other.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Understanding the subtle nuances of authorial intent is crucial for excelling in PTE reading. You're doing well by analyzing each option thoroughly!&lt;/p&gt;</t>
+          <t>&lt;p&gt;This question asks why the author mentions phonograph parlors. The paragraph uses them as the model for the later Kinetoscope arcades.&lt;/p&gt;
+&lt;ul&gt;
+&lt;li&gt;&lt;strong&gt;describe the model used to design Kinetoscope parlors (Correct)&lt;/strong&gt;&lt;p&gt;The first sentence says the Kinetoscope arcades were "modeled on phonograph parlors." The paragraph then explains that phonograph customers moved from one machine to another, and says Kinetoscope parlors functioned in a similar way. This is the direct reason the author discusses them.&lt;/p&gt;&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;explain Edison's financial success (Incorrect)&lt;/strong&gt;&lt;p&gt;The passage says phonograph parlors had been successful, but it does not explain the financial details of that success. The focus is the design model for Kinetoscope parlors.&lt;/p&gt;&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;contrast their operational modes and commercial focuses with those of Kinetoscope parlors (Incorrect)&lt;/strong&gt;&lt;p&gt;The paragraph does not contrast the operational modes. It says the Kinetoscope parlors functioned in a similar way. It also gives very little detail about the commercial focus of phonograph parlors, so this option overstates the comparison.&lt;/p&gt;&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;illustrate how much more technologically advanced Kinetoscope parlors were (Incorrect)&lt;/strong&gt;&lt;p&gt;The passage compares the parlor arrangement, not the technical advancement of one parlor type over the other.&lt;/p&gt;&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;emphasize that phonograph parlors were more profitable than Kinetoscope parlors (Incorrect)&lt;/strong&gt;&lt;p&gt;No profitability comparison is made between phonograph and Kinetoscope parlors.&lt;/p&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V1.8.1 - ROP Cohesion Feedback and Difficulty Filtering
</commit_message>
<xml_diff>
--- a/public/database/RMCMA/RMCMA/RMCMA.xlsx
+++ b/public/database/RMCMA/RMCMA/RMCMA.xlsx
@@ -854,31 +854,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. It's crucial in PTE Academic to carefully match the options to the exact information provided in the passage. We'll go through each statement to see if it aligns with the text.&lt;/p&gt;
-&lt;p&gt;Here's a detailed analysis:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Snow is formed from ice. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This statement is directly supported by the first sentence of the passage: "Snow is formed when temperatures are low and there is moisture - &lt;strong&gt;in the form of tiny ice crystals&lt;/strong&gt; - in the atmosphere." The passage clearly states that snow originates from these ice crystals, which are a form of ice. Therefore, this statement accurately reflects the information given.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Falling snow melts because of warm air around it. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage states, "The falling snow does begin to melt as soon as the temperature rises above freezing, but &lt;strong&gt;as the melting process begins, the air around the snowflake is cooled&lt;/strong&gt;." This contradicts the option. While snow melts when the ambient temperature rises above freezing, the passage explicitly says that the melting process itself *cools* the air immediately around the snowflake, rather than melting *because of* warm air around it. The initial cause is the general air temperature, but the effect on the immediate surroundings is cooling.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Subzero temperatures are required for snow to fall. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage directly refutes this. It states, "Precipitation falls as snow when the air temperature is below 2°C. &lt;strong&gt;It is a myth that it needs to be below zero to snow.&lt;/strong&gt; In fact the heaviest snowfalls tend to occur when the air temperature is between zero and 2°C." This clearly indicates that subzero temperatures are not a requirement for snow to fall.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Sleet develops at less than two degrees centigrade. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage states the opposite: "If the temperature is &lt;strong&gt;warmer than 2°C&lt;/strong&gt; then the snowflake will melt and fall as sleet rather than snow..." This means sleet forms *above* 2°C, not below it. Therefore, this statement is incorrect.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Dry snow falls in colder temperatures than wet snow. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage describes dry snow as falling through "dry, &lt;strong&gt;cool air&lt;/strong&gt;" and wet snow forming "When the temperature is &lt;strong&gt;slightly warmer than 0°C&lt;/strong&gt;". Since "cool air" generally implies temperatures at or below 0°C, and wet snow specifically forms when it's *slightly warmer than 0°C*, it logically follows that dry snow is associated with colder temperatures than wet snow. The passage draws a clear distinction in temperature conditions for these two types of snow.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! By carefully comparing each option to the specific details in the passage, you can confidently identify the correct answers in your PTE Academic exam.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Snow is formed from ice.&lt;/strong&gt; Selected. The passage says snow forms from moisture in the form of tiny ice crystals.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Falling snow melts because of warm air around it.&lt;/strong&gt; Not selected. The passage says falling snow begins to melt when the temperature rises above freezing, but it also says the air immediately around the snowflake is cooled as melting begins. The option is not a precise match.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Subzero temperatures are required for snow to fall.&lt;/strong&gt; Not selected. The passage directly says it is a myth that snow needs temperatures below zero.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Sleet develops at less than two degrees centigrade.&lt;/strong&gt; Not selected. The passage says sleet forms when the temperature is warmer than 2 degrees C, not less than 2 degrees C.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Dry snow falls in colder temperatures than wet snow.&lt;/strong&gt; Selected. The passage links dry snow with dry, cool air and wet snow with temperatures slightly warmer than 0 degrees C.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1288,8 +1264,8 @@
 ---
 Which of the following statements are true of Matthew Brady?
 ---
-[x] He was given permission to travel anywhere in the US.
-[x] He was able to give his photographers introductions to politicians.
+[x] He was given permission to travel anywhere with the Union armies.
+[x] He provided access to many leading generals and politicians.
 [] He took as many as seven thousand pictures of the war.
 [x] He was responsible for organizing a large number of photographers.
 [] Before the war he had been an amateur photographer.</t>
@@ -1297,34 +1273,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Understanding how to identify correct and incorrect information based on the passage is a crucial skill for the PTE Academic exam. We'll go through each option step-by-step.&lt;/p&gt;
-&lt;h3&gt;Explanation of Correct Options&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;strong&gt;He was given permission to travel anywhere in the US.&lt;/strong&gt;
-        &lt;p&gt;This statement is &lt;strong&gt;correct&lt;/strong&gt;. The passage explicitly states: "Lincoln granted him permission to travel anywhere with the Union armies". Since the Union armies were operating within the United States during the Civil War, this permission effectively allowed him to travel anywhere within the operational areas of the US where the Union forces were present. This is a reasonable interpretation of the scope of his travel.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;strong&gt;He was able to give his photographers introductions to politicians.&lt;/strong&gt;
-        &lt;p&gt;This statement is &lt;strong&gt;correct&lt;/strong&gt;. The passage mentions Brady's unique organizational skills, stating: "no one else could have organized the large army of photographers needed to cover the broad sweep of the war and provided access to many leading generals and politicians." This clearly indicates that Brady was instrumental in providing his team with access to important political figures, which would include introductions.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;strong&gt;He was responsible for organizing a large number of photographers.&lt;/strong&gt;
-        &lt;p&gt;This statement is &lt;strong&gt;correct&lt;/strong&gt;. The passage directly supports this by saying: "no one else could have organized the large army of photographers needed to cover the broad sweep of the war". This highlights his crucial role as an organizer and manager of a vast photographic operation.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Explanation of Incorrect Options&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;strong&gt;He took as many as seven thousand pictures of the war.&lt;/strong&gt;
-        &lt;p&gt;This statement is &lt;strong&gt;incorrect&lt;/strong&gt;. The passage directly contradicts this by stating: "he had hundreds of assistants, and it's even possible that he didn't take any of the 7,000 pictures that were marketed under his name." While 7,000 pictures were associated with his name, the passage explicitly questions whether he personally took any of them, let alone all of them.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;strong&gt;Before the war he had been an amateur photographer.&lt;/strong&gt;
-        &lt;p&gt;This statement is &lt;strong&gt;incorrect&lt;/strong&gt;. The passage describes Matthew Brady as "a well-known portrait photographer" in 1861, which was the start of the Civil War. Being "well-known" in a specific field implies professionalism, not amateur status. In contrast, the passage mentions Roger Fenton as an "amateur photographer," clearly distinguishing him from Brady.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! By carefully reading and cross-referencing each option with the text, you can confidently identify the correct answers in your PTE Academic exam.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;He was given permission to travel anywhere with the Union armies.&lt;/strong&gt; Selected. The passage states that Lincoln granted Brady permission to travel anywhere with the Union armies.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;He provided access to many leading generals and politicians.&lt;/strong&gt; Selected. The passage says Brady provided access to many leading generals and politicians.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;He took as many as seven thousand pictures of the war.&lt;/strong&gt; Not selected. The passage says it is possible Brady did not take any of the 7,000 pictures marketed under his name.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;He was responsible for organizing a large number of photographers.&lt;/strong&gt; Selected. The passage says no one else could have organized the large army of photographers needed to cover the war.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Before the war he had been an amateur photographer.&lt;/strong&gt; Not selected. The passage describes Brady as a well-known portrait photographer; the amateur photographer mentioned is Roger Fenton.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1455,9 +1404,9 @@
         <is>
           <t>Sensitivity to physical laws is thus an important consideration for the maker of applied-art objects. It is often taken for granted that this is also true for the maker of fine-art objects. This assumption misses a significant difference between the two disciplines. Fine-art objects are not constrained by the laws of physics in the same way that applied-art objects are. Because their primary purpose is not functional, they are only limited in terms of the materials used to make them. Sculptures must, for example, be stable, which requires an understanding of the properties of mass, weight distribution, and stress. Paintings must have rigid stretchers so that the canvas will be taut, and the paint must not deteriorate, crack, or discolor. These are problems that must be overcome by the artist because they tend to intrude upon his or her conception of the work. For example, in the early Italian Renaissance, bronze statues of horses with a raised foreleg usually had a cannonball under that hoof. This was done because the cannonball was needed to support the weight of the leg. In other words, the demands of the laws of physics, not the sculptor's aesthetic intentions, placed the ball there. That this device was a necessary structural compromise is clear from the fact that the cannonball quickly disappeared when sculptors learned how to strengthen the internal structure of a statue with iron braces (iron being much stronger than bronze).
 ---
-According to paragraph, sculptors in the Italian Renaissance stopped using cannonballs in bronze statues of horses because
----
-[x] they began using a material that much stronger
+According to the paragraph, sculptors in the Italian Renaissance stopped using cannonballs in bronze statues of horses because
+---
+[x] they began using a much stronger material
 [x] they found a way to strengthen the statues internally
 [] the aesthetic tastes of the public had changed over time
 [] the cannonballs added too much weight to the statues</t>
@@ -1465,23 +1414,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this question and passage together to understand why certain options are correct and others are not. This is a great way to improve your reading comprehension and analytical skills for the PTE Academic exam.&lt;/p&gt;
-&lt;p&gt;The question asks why sculptors in the Italian Renaissance stopped using cannonballs in bronze statues of horses. We need to find the specific reason mentioned in the passage for the disappearance of these cannonballs.&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;they began using a material that much stronger (Correct)&lt;/strong&gt;
-        &lt;p&gt;This option is &lt;strong&gt;correct&lt;/strong&gt;. The passage explicitly states: "That this device was a necessary structural compromise is clear from the fact that the cannonball quickly disappeared when sculptors learned how to strengthen the internal structure of a statue with iron braces (&lt;strong&gt;iron being much stronger than bronze&lt;/strong&gt;)." This sentence directly tells us that the use of a stronger material (iron) was the key factor in eliminating the need for cannonballs.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;&lt;strong&gt;they found a way to strengthen the statues internally (Correct)&lt;/strong&gt;
-        &lt;p&gt;This option is also &lt;strong&gt;correct&lt;/strong&gt;. The passage states: "the cannonball quickly disappeared when sculptors learned how to &lt;strong&gt;strengthen the internal structure of a statue with iron braces&lt;/strong&gt;". This directly supports the idea that sculptors developed a method to reinforce the statue from within, making the external cannonball unnecessary. The internal strengthening was achieved by using iron braces, which links to the previous correct option.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;&lt;strong&gt;the aesthetic tastes of the public had changed over time (Incorrect)&lt;/strong&gt;
-        &lt;p&gt;This option is &lt;strong&gt;incorrect&lt;/strong&gt;. The passage clearly states that the cannonball was a "necessary structural compromise" and that "the demands of the laws of physics, not the sculptor's aesthetic intentions, placed the ball there." This indicates that the cannonball was a functional necessity, not an aesthetic choice. Therefore, its removal was due to overcoming a physical constraint, not a change in public taste. The passage does not mention anything about changing aesthetic tastes.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;&lt;strong&gt;the cannonballs added too much weight to the statues (Incorrect)&lt;/strong&gt;
-        &lt;p&gt;This option is &lt;strong&gt;incorrect&lt;/strong&gt;. The passage states the opposite: "bronze statues of horses with a raised foreleg usually had a cannonball under that hoof. This was done because the cannonball was &lt;strong&gt;needed to support the weight of the leg&lt;/strong&gt;." The cannonball was a solution to a weight distribution problem, providing necessary support, not an additional burden of excessive weight. The problem was the *lack of internal strength* to support the raised leg, not that the cannonball itself was too heavy.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Understanding how to pinpoint specific details and distinguish them from unsupported claims is crucial for success in the PTE Academic reading section.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;they began using a much stronger material&lt;/strong&gt; Selected. The passage explains that sculptors used iron braces and notes that iron is much stronger than bronze.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;they found a way to strengthen the statues internally&lt;/strong&gt; Selected. The passage says the cannonball disappeared when sculptors learned how to strengthen the internal structure of the statue.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;the aesthetic tastes of the public had changed over time&lt;/strong&gt; Not selected. The passage says the cannonball was required by physical structure, not aesthetic taste.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;the cannonballs added too much weight to the statues&lt;/strong&gt; Not selected. The cannonball supported the raised leg; the passage does not say it was removed because it added too much weight.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1545,45 +1478,17 @@
         <is>
           <t>The fossil consists of a complete skull of an archaeocyte, an extinct group of ancestors of modern cetaceans. Although limited to a skull, the Pakicetus fossil provides precious details on the origins of cetaceans. The skull is cetacean-like but its jawbones lack the enlarged space that is filled with fat or oil and used for receiving underwater sound in modern whales. Pakicetus probably detected sound through the ear opening as in land mammals. The skull also lacks a blowhole, another cetacean adaptation for diving. Other features, however, show experts that Pakicetus is a transitional form between a group of extinct flesh-eating mammals, the mesonychids, and cetaceans. It has been suggested that Pakicetus fed on fish in shallow water and was not yet adapted for life in the open ocean. It probably bred and gave birth on land.
 ---
-Pakicetus and modern cetaceans have similar ____ .
+Pakicetus and modern cetaceans have similar ____.
 ---
 [] hearing structures
 [] adaptations for diving
 [x] skull shapes
-[x] feeding locations</t>
+[] feeding locations</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this question and passage to understand why certain options are correct and others are not. This will help you sharpen your reading comprehension skills for the PTE Academic exam.&lt;/p&gt;
-&lt;p&gt;The question asks us to identify &lt;strong&gt;similarities&lt;/strong&gt; between &lt;strong&gt;Pakicetus&lt;/strong&gt; and &lt;strong&gt;modern cetaceans&lt;/strong&gt; based on the provided text.&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Correct Option: skull shapes&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage explicitly states, &lt;strong&gt;"The skull is cetacean-like..."&lt;/strong&gt; This phrase directly indicates a similarity in the overall shape or general appearance of the skull between Pakicetus and modern cetaceans. Even though there are specific differences in features like jawbones for hearing or the presence of a blowhole, the fundamental form of the skull is noted as similar.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Correct Option: feeding locations&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage states, &lt;strong&gt;"It has been suggested that Pakicetus fed on fish in shallow water..."&lt;/strong&gt; This tells us that Pakicetus obtained its food from an aquatic environment. While the passage also notes Pakicetus "was not yet adapted for life in the open ocean" (implying modern cetaceans are), the fundamental similarity in "feeding locations" is that both Pakicetus (as an ancestor) and modern cetaceans obtain their food from &lt;strong&gt;aquatic environments&lt;/strong&gt;. "Shallow water" is a specific type of aquatic feeding location, and modern cetaceans, being fully aquatic, also feed in various aquatic locations. Therefore, the general nature of their feeding locations being aquatic is a shared characteristic.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Incorrect Option: hearing structures&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage highlights significant differences in hearing structures. It states, &lt;strong&gt;"its jawbones lack the enlarged space that is filled with fat or oil and used for receiving underwater sound in modern whales."&lt;/strong&gt; It further clarifies, &lt;strong&gt;"Pakicetus probably detected sound through the ear opening as in land mammals."&lt;/strong&gt; This clearly shows that their hearing mechanisms and structures were different, not similar.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Incorrect Option: adaptations for diving&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage explicitly states that Pakicetus *lacked* adaptations for diving that modern cetaceans possess. It mentions, &lt;strong&gt;"The skull also lacks a blowhole, another cetacean adaptation for diving."&lt;/strong&gt; Additionally, it notes Pakicetus &lt;strong&gt;"was not yet adapted for life in the open ocean,"&lt;/strong&gt; which implies a lack of adaptations for a fully aquatic, diving lifestyle typical of modern cetaceans. Therefore, this is a point of difference, not similarity.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Focusing on direct textual evidence and careful interpretation is key to mastering these types of questions.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;hearing structures&lt;/strong&gt; Not selected. The passage contrasts Pakicetus with modern whales by saying it lacked the enlarged jawbone space used for underwater sound.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;adaptations for diving&lt;/strong&gt; Not selected. The passage says Pakicetus lacked a blowhole, a cetacean adaptation for diving.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;skull shapes&lt;/strong&gt; Selected. The passage directly states that the skull is cetacean-like.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;feeding locations&lt;/strong&gt; Not selected. The passage says Pakicetus fed in shallow water and was not yet adapted for life in the open ocean; it does not directly support similar feeding locations.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1604,44 +1509,14 @@
 ---
 [] Fossil legs of early whales are a rare find.
 [x] The legs provided important information about the evolution of cetaceans.
-[x] The discovery allowed scientists to reconstruct a complete evolution of the whale.
+[] The discovery allowed scientists to reconstruct a complete evolution of the whale.
 [] Until that time, only the front legs of early whales had been discovered.
 [] The scientists took more than a decade to find the fossil.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! This is a fantastic question that really tests your ability to understand the author's intent and the significance of details in a passage. Let's break down why the author used "luckily" and evaluate each option carefully.&lt;/p&gt;
-&lt;p&gt;The word "luckily" implies that the presence of the hind legs in the fossil was a fortunate circumstance because it yielded valuable information or allowed for a significant understanding that might otherwise have been missed. We need to look at what the passage says *after* mentioning the hind legs to understand their importance.&lt;/p&gt;
-&lt;p&gt;The passage states: "The fossil luckily includes a good portion of the hind legs. The legs were strong and ended in long feet very much like those of a modern pinniped. The legs were certainly functional both on land and at sea... The large hind legs were used for propulsion in water. On land... Ambulocetus may have moved around very much like a modern sea lion. It was undoubtedly a whale that linked life on land with life at sea."&lt;/p&gt;
-&lt;p&gt;This entire description highlights the crucial information these hind legs provided about the whale's transitional lifestyle and its evolutionary role.&lt;/p&gt;
-&lt;h3&gt;Correct Options Explained:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The legs provided important information about the evolution of cetaceans.&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why this is correct:&lt;/strong&gt; This option directly reflects the passage's emphasis. Immediately after "luckily," the text details *what* the legs revealed: they were "functional both on land and at sea," used for "propulsion in water," and allowed Ambulocetus to move "like a modern sea lion" on land. All this information is vital for understanding how whales evolved from land-dwelling ancestors to fully aquatic creatures. The hind legs were the key evidence for this transitional phase, making their discovery "lucky" because they provided such critical evolutionary insights.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The discovery allowed scientists to reconstruct a complete evolution of the whale.&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why this is correct:&lt;/strong&gt; While "complete evolution" might seem like a strong claim for a single fossil, the passage concludes by stating, "It was undoubtedly a whale that linked life on land with life at sea." This statement signifies a monumental breakthrough in understanding a crucial phase of whale evolution – the transition from land to sea. The presence of functional hind legs was the primary evidence that allowed scientists to understand and reconstruct this vital link, thereby making the overall picture of whale evolution much more complete. Without these legs, this critical piece of the evolutionary puzzle would have been missing or much harder to piece together. Therefore, the discovery was "lucky" because it enabled this significant reconstruction.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Incorrect Options Explained:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Fossil legs of early whales are a rare find.&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why this is incorrect:&lt;/strong&gt; The passage does not state that fossil legs of early whales are generally rare. While it might be true in the broader field of paleontology, the text itself does not provide this information as the reason for using "luckily." The author uses "luckily" to emphasize the *utility* and *significance* of *these specific* hind legs in understanding Ambulocetus's lifestyle and evolutionary role, not their general rarity in the fossil record.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Until that time, only the front legs of early whales had been discovered.&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why this is incorrect:&lt;/strong&gt; The passage makes no mention of previous discoveries of front legs or the absence of hind legs in other early whale fossils. This option introduces information that is not supported or even hinted at in the provided text. We must base our answers solely on the information given in the passage.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The scientists took more than a decade to find the fossil.&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why this is incorrect:&lt;/strong&gt; The passage states that the find was "reported in 1994" but provides no information whatsoever about how long it took the scientists to discover the fossil. The duration of the search is irrelevant to why the author used the word "luckily" in reference to the hind legs being present.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Understanding the nuances of word choice and how details contribute to the main idea is key in PTE Reading. You're doing well by dissecting each option against the passage.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Fossil legs of early whales are a rare find.&lt;/strong&gt; Not selected. The passage does not state that fossil legs of early whales are generally rare.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The legs provided important information about the evolution of cetaceans.&lt;/strong&gt; Selected. The passage uses the hind legs to explain movement on land and in water and says Ambulocetus linked life on land with life at sea.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The discovery allowed scientists to reconstruct a complete evolution of the whale.&lt;/strong&gt; Not selected. The passage supports an important transitional link, not a complete reconstruction of whale evolution.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Until that time, only the front legs of early whales had been discovered.&lt;/strong&gt; Not selected. The passage does not say that only front legs had been discovered before.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The scientists took more than a decade to find the fossil.&lt;/strong&gt; Not selected. The passage does not mention how long scientists took to find the fossil.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1720,14 +1595,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>&lt;p&gt;This question asks why the author mentions phonograph parlors. The paragraph uses them as the model for the later Kinetoscope arcades.&lt;/p&gt;
-&lt;ul&gt;
-&lt;li&gt;&lt;strong&gt;describe the model used to design Kinetoscope parlors (Correct)&lt;/strong&gt;&lt;p&gt;The first sentence says the Kinetoscope arcades were "modeled on phonograph parlors." The paragraph then explains that phonograph customers moved from one machine to another, and says Kinetoscope parlors functioned in a similar way. This is the direct reason the author discusses them.&lt;/p&gt;&lt;/li&gt;
-&lt;li&gt;&lt;strong&gt;explain Edison's financial success (Incorrect)&lt;/strong&gt;&lt;p&gt;The passage says phonograph parlors had been successful, but it does not explain the financial details of that success. The focus is the design model for Kinetoscope parlors.&lt;/p&gt;&lt;/li&gt;
-&lt;li&gt;&lt;strong&gt;contrast their operational modes and commercial focuses with those of Kinetoscope parlors (Incorrect)&lt;/strong&gt;&lt;p&gt;The paragraph does not contrast the operational modes. It says the Kinetoscope parlors functioned in a similar way. It also gives very little detail about the commercial focus of phonograph parlors, so this option overstates the comparison.&lt;/p&gt;&lt;/li&gt;
-&lt;li&gt;&lt;strong&gt;illustrate how much more technologically advanced Kinetoscope parlors were (Incorrect)&lt;/strong&gt;&lt;p&gt;The passage compares the parlor arrangement, not the technical advancement of one parlor type over the other.&lt;/p&gt;&lt;/li&gt;
-&lt;li&gt;&lt;strong&gt;emphasize that phonograph parlors were more profitable than Kinetoscope parlors (Incorrect)&lt;/strong&gt;&lt;p&gt;No profitability comparison is made between phonograph and Kinetoscope parlors.&lt;/p&gt;&lt;/li&gt;
-&lt;/ul&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;explain Edison&amp;#x27;s financial success&lt;/strong&gt; Not selected. The paragraph focuses on the business model for Kinetoscope parlors, not Edison&amp;#x27;s overall financial success.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;describe the model used to design Kinetoscope parlors&lt;/strong&gt; Selected. The passage states that Kinetoscope arcades were modeled on phonograph parlors.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;contrast their operational modes and commercial focuses with those of Kinetoscope parlors&lt;/strong&gt; Not selected. The passage says Kinetoscope parlors functioned in a similar way; it does not present a contrast.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;illustrate how much more technologically advanced Kinetoscope parlors were&lt;/strong&gt; Not selected. The passage does not compare the technological advancement of the two kinds of parlors.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;emphasize that phonograph parlors were more profitable than Kinetoscope parlors&lt;/strong&gt; Not selected. The passage says phonograph parlors had proven successful, but it does not compare profitability.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1847,37 +1715,15 @@
 In the paragraph, the author includes the quotation from a mill worker in order to
 ---
 [x] support the idea that it was difficult for workers to adjust to working in factories.
-[] to show that workers sometimes quit because of the loud noise made by factory machinery.
-[x] argue that clocks were more useful in factories than ever before.
+[] show that workers sometimes quit because of the loud noise made by factory machinery.
+[] argue that clocks were more useful in factories than ever before.
 [] emphasize that factories were most successful when workers revealed their complaints.
 [] emphasize that factory workers enjoyed the structured routine imposed by the bell.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this question and passage together to understand why certain options are correct and others are not. This will help you develop a strong analytical approach for your PTE Academic reading tasks.&lt;/p&gt;
-&lt;h3&gt;Correct Options Explained:&lt;/h3&gt;
-&lt;h4&gt;1. support the idea that it was difficult for workers to adjust to working in factories.&lt;/h4&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; This option is strongly supported by the passage. Immediately preceding the quotation, the text states, "&lt;strong&gt;The first generation to experience these changes did not adopt the new attitudes easily.&lt;/strong&gt; The factory clock became the symbol of the new work rules." The mill worker's complaint about "obedience to the ding-dong of the bell-just as though we are so many living machines" serves as a powerful, firsthand illustration of this difficulty. The worker's feeling of being dehumanized and controlled by the bell, to the point of quitting, directly demonstrates the profound challenges and negative experiences workers faced in adjusting to the strict, regimented, and impersonal factory environment. The author includes this quote precisely to provide concrete evidence of the workers' struggle to adapt.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h4&gt;2. argue that clocks were more useful in factories than ever before.&lt;/h4&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; While the quote is a complaint, it implicitly highlights the immense utility of the clock/bell from the factory's perspective. The passage explains that "The new methods of doing business involved a new and stricter sense of time. Factory life necessitated a more regimented schedule, where work began at the sound of a bell and workers kept machines going at a constant pace." The fact that the bell had such a pervasive and controlling influence on the worker, making them feel like a "living machine," underscores its critical role in enforcing this new, highly efficient, and disciplined work regimen. The author uses the worker's intense reaction to demonstrate just how indispensable and effective (i.e., useful) the clock had become in managing and optimizing factory operations, even if it was at the expense of worker autonomy and well-being. The complaint, in its very nature, reveals the clock's powerful and central function in the industrial system.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Incorrect Options Explained:&lt;/h3&gt;
-&lt;h4&gt;1. to show that workers sometimes quit because of the loud noise made by factory machinery.&lt;/h4&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; This option misinterprets the specific content of the quotation. The worker complains about the "&lt;strong&gt;ding-dong of the bell&lt;/strong&gt;" and the feeling of being a "living machine" due to its command, which symbolizes the strict, regimented schedule and loss of personal freedom. The quote does not mention or imply that the worker quit due to the general "loud noise made by factory machinery." The focus is on the oppressive control of time and schedule, not auditory discomfort from machines.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h4&gt;2. emphasize that factories were most successful when workers revealed their complaints.&lt;/h4&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; This option presents a cause-and-effect relationship that is not supported by the passage. The passage describes the negative impact of industrialization on workers, leading to complaints and a sense of decline in status. The worker in the quote actually "quit," which is a negative outcome for the factory (loss of labor), not a factor contributing to its success. The author includes the complaint to illustrate worker dissatisfaction and difficulty, not to suggest that complaints lead to factory prosperity.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h4&gt;3. emphasize that factory workers enjoyed the structured routine imposed by the bell.&lt;/h4&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; This option directly contradicts the clear sentiment expressed in the quotation and the overall context of the passage. The worker explicitly complains about "obedience to the ding-dong of the bell" and feeling "just as though we are so many living machines," which clearly indicates *dislike* and *resentment*, not enjoyment. Furthermore, the passage states that the first generation of workers "did not adopt the new attitudes easily," reinforcing the idea that the structured routine was a source of difficulty, not pleasure.&lt;/li&gt;
-&lt;/ul&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;support the idea that it was difficult for workers to adjust to working in factories.&lt;/strong&gt; Selected. The quote complains about obedience to the bell and being treated like living machines, showing the difficulty of adjusting to factory discipline.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;show that workers sometimes quit because of the loud noise made by factory machinery.&lt;/strong&gt; Not selected. The quote mentions the bell, not loud machinery, and the complaint is about loss of freedom.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;argue that clocks were more useful in factories than ever before.&lt;/strong&gt; Not selected. The quote shows the human cost of the factory clock; it does not argue that clocks were useful.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;emphasize that factories were most successful when workers revealed their complaints.&lt;/strong&gt; Not selected. The passage does not connect worker complaints to factory success.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;emphasize that factory workers enjoyed the structured routine imposed by the bell.&lt;/strong&gt; Not selected. The worker complains about the bell and says he left because he could not give up freedom.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -1997,40 +1843,12 @@
 [] The Democratic Party's main source of support
 [x] The people that Democrats claimed were unfairly becoming rich
 [] The people most interested in a return to a simple agrarian republic
-[x] One of the groups might be not in favor of Whig party and Democrats</t>
+[] A group that might not favor either the Whig Party or the Democratic Party</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Understanding how to identify correct and incorrect options is a crucial skill for the PTE Academic test. We'll go through each choice carefully.&lt;/p&gt;
-&lt;p&gt;The passage describes the Democratic Party's views during Jackson's second term, particularly their stance on bankers and investors.&lt;/p&gt;
-&lt;p&gt;&lt;strong&gt;Passage Snippet for Reference:&lt;/strong&gt;&lt;br&gt;
-"The Democrats tended to view society as a continuing conflict between 'the people'—farmers, planters, and workers—and a set of greedy aristocrats. This 'paper money aristocracy' of bankers and investors manipulated the banking system for their own profit, Democrats claimed, and sapped the nation's virtue by encouraging speculation and the desire for sudden, unearned wealth."&lt;/p&gt;
-&lt;h3&gt;Analysis of Options:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The people that Democrats claimed were unfairly becoming rich (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is clearly supported by the passage. The text explicitly states that Democrats viewed bankers and investors as a "'paper money aristocracy' who manipulated the banking system for their own profit" and encouraged "the desire for sudden, unearned wealth." The phrase "unearned wealth" directly indicates that Democrats believed these individuals were becoming rich unfairly. This aligns perfectly with the question asking what bankers and investors were an example of in the Democrats' view.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;One of the groups might be not in favor of Whig party and Democrats (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option requires a bit more inference, but we can see why it might be considered correct.
-            &lt;ul&gt;
-                &lt;li&gt;&lt;strong&gt;Not in favor of Democrats:&lt;/strong&gt; The passage clearly states that Democrats viewed bankers and investors as "greedy aristocrats" who "manipulated the banking system for their own profit." Given such strong negative characterization and opposition from the Democrats, it's highly probable that bankers and investors would not be in favor of the Democratic Party.&lt;/li&gt;
-                &lt;li&gt;&lt;strong&gt;Not in favor of Whig party:&lt;/strong&gt; The passage mentions that "Whigs and Democrats held different attitudes toward the changes brought about by the market, banks, and commerce." While the passage doesn't detail the Whigs' specific stance on bankers and investors, the fact that there were "different attitudes" suggests that neither party might perfectly align with all the interests of bankers and investors. Even if Whigs were generally more pro-business, specific policies or aspects of their platform might not have been universally favored by all bankers and investors. Therefore, it's plausible that some within this group might not have been in favor of *both* parties, seeking their own specific interests. This makes it a possible, though less direct, inference than the first correct option.&lt;/li&gt;
-            &lt;/ul&gt;
-        &lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The Democratic Party's main source of support (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option directly contradicts the information in the passage. The Democrats viewed bankers and investors as "greedy aristocrats" and their opponents, not as a source of support. The passage highlights a conflict between "the people" (farmers, planters, workers) and this "paper money aristocracy," clearly positioning bankers and investors as adversaries, not allies, of the Democratic Party.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The people most interested in a return to a simple agrarian republic (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is incorrect because the passage attributes the desire for a "simple agrarian republic" to the Democrats, not to bankers and investors. The text states, "The Democrats wanted the rewards of the market without sacrificing the features of a simple agrarian republic." Bankers and investors, described as manipulating the banking system and encouraging speculation, represent the very forces of market change and complex dealings that the Democrats wished to temper, not the group interested in an agrarian ideal.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! By carefully comparing each option to the specific details and implications in the passage, you can confidently choose the best answers.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The Democratic Party&amp;#x27;s main source of support&lt;/strong&gt; Not selected. The passage lists farmers, planters, and workers as the people in the Democrats&amp;#x27; social conflict, not bankers and investors as their support base.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The people that Democrats claimed were unfairly becoming rich&lt;/strong&gt; Selected. The passage says Democrats claimed bankers and investors manipulated the banking system for profit and encouraged unearned wealth.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The people most interested in a return to a simple agrarian republic&lt;/strong&gt; Not selected. The passage says Democrats wanted to preserve features of a simple agrarian republic; it does not attribute this interest to bankers and investors.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;A group that might not favor either the Whig Party or the Democratic Party&lt;/strong&gt; Not selected. The passage does not discuss bankers&amp;#x27; and investors&amp;#x27; party preferences.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -2285,49 +2103,12 @@
 [] Artists painted pictures on both walls and bones.
 [] Artists ground them into a fine powder to make paint.
 [x] Artists developed special techniques for painting the walls.
-[x] Bones were not only relate to food.</t>
+[x] The bones were used for more than food-related purposes.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello! Let's break down this question and the options to understand why some are correct and others are not. This is a great way to improve your reading comprehension and critical thinking skills for the PTE Academic test.&lt;/p&gt;
-&lt;p&gt;The question asks: &lt;strong&gt;What are the bones found in the Lascaux caves believed to indicate?&lt;/strong&gt;&lt;/p&gt;
-&lt;p&gt;We need to focus on the part of the passage that discusses the bones and their purpose:&lt;/p&gt;
-&lt;p&gt;&lt;em&gt;"Methods of applying color varied: some colors were brushed or smeared on rock surfaces and others were blown or sprayed. It is possible that tubes made from animal bones were used for spraying because hollow bones, some stained with pigment, have been found nearby."&lt;/em&gt;&lt;/p&gt;
-&lt;p&gt;Let's analyze each option:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The subjects the artists painted are varied. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; While the passage does mention a variety of animals painted ("bulls, wild horses, reindeer, bison, and mammoths"), this statement describes the *content* or *themes* of the paintings. The question specifically asks what the *bones* indicate. The bones are linked to the *method* of painting, not the subjects. Therefore, this option is irrelevant to the specific question about the bones' significance.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Artists painted pictures on both walls and bones. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; The passage states that paintings were on "rock surfaces" (walls). It mentions "hollow bones, some stained with pigment," which means there was paint *on* the bones. However, this does not imply that artists used the bones *as a canvas* to create pictures on them. Instead, the pigment on the bones is presented as evidence that the bones were used *as tools* for applying paint (specifically for spraying). This option misinterprets the role of the bones.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Artists ground them into a fine powder to make paint. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; The passage clearly states the origin of the paint colors: "Scientific analysis reveals that the colors were derived from ocher and other iron oxides ground into a fine powder." It explicitly attributes the paint powder to minerals like ocher and iron oxides, not to bones. The bones are mentioned as potential *tools for applying* the paint, not as a source material for the paint itself. This option directly contradicts the information provided in the passage.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Artists developed special techniques for painting the walls. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; The passage describes various application methods: "some colors were brushed or smeared on rock surfaces and others were blown or sprayed." It then directly connects the bones to one of these methods: "It is possible that tubes made from animal bones were used for spraying because hollow bones, some stained with pigment, have been found nearby." The discovery of these bones, stained with pigment, strongly suggests that ancient artists employed a sophisticated technique like spraying, which goes beyond simple brushing or smearing. Thus, the bones are evidence that these special painting techniques were developed and used.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Bones were not only relate to food. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; In prehistoric contexts, animal bones are primarily associated with sustenance – as remnants of hunted animals consumed for food. However, the passage presents a different, non-food-related use for these bones: "It is possible that tubes made from animal bones were used for spraying because hollow bones, some stained with pigment, have been found nearby." This discovery suggests that the bones served a purpose beyond just being food waste or tools for basic survival. They were repurposed as instruments for artistic creation, indicating a more complex and varied utility for animal bones in that era. This option highlights that their function extended beyond the most common assumption.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Understanding how to connect specific details in the passage to the question asked is a crucial skill for the PTE Academic test.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The subjects the artists painted are varied.&lt;/strong&gt; Not selected. The passage does list several animals, but the bones are discussed as possible tools for applying pigment, not as evidence of subject variety.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Artists painted pictures on both walls and bones.&lt;/strong&gt; Not selected. The passage says bones were stained with pigment and may have been used as tubes; it does not say pictures were painted on bones.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Artists ground them into a fine powder to make paint.&lt;/strong&gt; Not selected. The passage says ocher and iron oxides were ground into powder, not the bones.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Artists developed special techniques for painting the walls.&lt;/strong&gt; Selected. The stained hollow bones may have been used as tubes for spraying color, which supports a special painting technique.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The bones were used for more than food-related purposes.&lt;/strong&gt; Selected. Because the bones were stained with pigment and may have been used for spraying, the passage suggests they were not only food remains.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -2406,42 +2187,13 @@
 ---
 [] Farms using windmills to pump water
 [] Research centers exploring the uses of wind
-[x] Types of power plant common in Denmark and California
+[] Types of power plant common in Denmark and California
 [x] Collections of wind turbines producing electric power</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this question together to help you master your PTE Academic reading skills. Understanding how to identify direct evidence in a passage is crucial for these types of questions.&lt;/p&gt;
-&lt;p&gt;The question asks us to identify the best explanation for the term "wind farms" based *only* on the provided paragraph. This means we must stick strictly to the information given and not bring in outside knowledge.&lt;/p&gt;
-&lt;h3&gt;Analysis of the Passage:&lt;/h3&gt;
-&lt;p&gt;The passage states:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;"Since 1980, the use of wind to produce electricity has been growing rapidly." (This tells us the purpose of wind use).&lt;/li&gt;
-    &lt;li&gt;"In 1994 there were nearly 20,000 wind turbines worldwide, most grouped in clusters called wind farms that collectively produced 3,000 megawatts of electricity." (This is the key sentence defining and describing wind farms).&lt;/li&gt;
-    &lt;li&gt;"Most were in Denmark... and California..." (This tells us where they are common).&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Evaluation of Options:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Farms using windmills to pump water (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is incorrect because the passage explicitly states that wind is used "to produce electricity." There is no mention of windmills being used to pump water anywhere in the text. This option introduces information that is not supported by the passage and contradicts the stated purpose of wind energy in this context.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Research centers exploring the uses of wind (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is incorrect because the passage describes wind farms as operational entities that are "producing 3,000 megawatts of electricity," not as research centers. The text focuses on the *production* of electricity, not the *exploration* of new uses for wind. There is no mention of research or experimentation.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Types of power plant common in Denmark and California (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is correct because the passage states that wind farms "collectively produced 3,000 megawatts of electricity," which directly implies they are facilities for generating power, much like a power plant. Furthermore, the passage explicitly mentions that "Most were in Denmark (which got 3 percent of its electricity from wind turbines) and California (where 17,000 machines produced 1 percent of the state's electricity...)." This clearly indicates their prevalence in these locations as electricity-producing installations.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Collections of wind turbines producing electric power (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is also correct and is arguably the most direct explanation. The passage states, "...most grouped in clusters called wind farms that collectively produced 3,000 megawatts of electricity." The word "clusters" is synonymous with "collections," and "produced... electricity" directly matches "producing electric power." This option provides a clear and concise definition directly from the text.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Key Takeaway:&lt;/h3&gt;
-&lt;p&gt;Both "Types of power plant common in Denmark and California" and "Collections of wind turbines producing electric power" are correct based on the passage. The question asks for the "best explains," and often in PTE, there might be multiple correct statements, but one is more directly supported or comprehensive. In this case, the passage directly defines wind farms as "clusters" of turbines that "produced electricity," making "Collections of wind turbines producing electric power" a very strong and direct explanation. The other correct option describes a characteristic and location of these power-producing entities. Both accurately reflect information in the text.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Farms using windmills to pump water&lt;/strong&gt; Not selected. The paragraph is about wind turbines producing electricity, not pumping water.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Research centers exploring the uses of wind&lt;/strong&gt; Not selected. The paragraph defines wind farms as clusters of turbines, not research centers.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Types of power plant common in Denmark and California&lt;/strong&gt; Not selected. Denmark and California are locations where many wind turbines were found, but this does not best define the term wind farms.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Collections of wind turbines producing electric power&lt;/strong&gt; Selected. The passage says turbines were grouped in clusters called wind farms and collectively produced electricity.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -2856,28 +2608,12 @@
 [x] It presented some works that were not by Fuller.
 [] It featured performances by prominent male as well as female dancers.
 [] It became a famous school that is still named in honor of Fuller.
-[x] The passage does not tell whether It ceased to operate as a theater after Fuller died.</t>
+[] The passage does not tell whether it ceased to operate as a theater after Fuller died.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this question and the options to understand why some are correct and others are not. This is a great way to sharpen your reading comprehension skills for the PTE Academic test.&lt;/p&gt;
-&lt;p&gt;The question asks what was true of Fuller's theater at the Paris Exposition, according to the paragraph. We need to find direct evidence or strong implications from the text for each option.&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;&lt;p&gt;It presented some works that were not by Fuller. (Correct)&lt;/p&gt;&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This option is directly supported by the first sentence of the passage: "At the Paris Exposition in 1900, Fuller had her own theater, where, &lt;strong&gt;in addition to her own dances, she presented pantomimes by the Japanese actress Sada Yocco.&lt;/strong&gt;" The phrase "in addition to her own dances" clearly indicates that other works, specifically Sada Yocco's pantomimes, were also presented. These pantomimes were "works that were not by Fuller."&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;&lt;strong&gt;&lt;p&gt;It featured performances by prominent male as well as female dancers. (Incorrect)&lt;/p&gt;&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage states, "&lt;strong&gt;She assembled an all-female company at this time&lt;/strong&gt; and established a school around 1908..." While this refers to her company, the context of her performances at the theater strongly implies that her company, which was all-female, would be performing. There is no mention of male dancers performing at her theater. In fact, the mention of an "all-female company" suggests the opposite of this option.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;&lt;strong&gt;&lt;p&gt;It became a famous school that is still named in honor of Fuller. (Incorrect)&lt;/p&gt;&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage mentions that Fuller "established a school around 1908," but it explicitly states that "&lt;strong&gt;neither survived her.&lt;/strong&gt;" This means the school did not continue to exist after her death, let alone become "still named in honor of Fuller." Furthermore, the school was established "around 1908," which is eight years after the Paris Exposition in 1900, so the theater at the exposition itself did not become this school.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;&lt;strong&gt;&lt;p&gt;The passage does not tell whether It ceased to operate as a theater after Fuller died. (Correct)&lt;/p&gt;&lt;/strong&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The question specifically asks about Fuller's theater *at the Paris Exposition*. The passage states this exposition was in 1900. Expositions are typically temporary events. While the passage mentions that Fuller's *school* and *company* did not survive her, it provides no information whatsoever about the long-term fate or cessation of operation of the *specific theater at the Paris Exposition* after Fuller's death. We can infer that a temporary exposition theater would likely cease to exist after the exposition, but the passage does not explicitly state this, nor does it link its cessation to Fuller's death. Therefore, the passage is silent on this particular detail.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Understanding how to find direct evidence and identify what is *not* stated in the passage is crucial for success in reading comprehension tasks.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;It presented some works that were not by Fuller.&lt;/strong&gt; Selected. The passage says Fuller presented pantomimes by the Japanese actress Sada Yocco in addition to her own dances.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;It featured performances by prominent male as well as female dancers.&lt;/strong&gt; Not selected. The passage mentions an all-female company and does not mention male dancers performing there.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;It became a famous school that is still named in honor of Fuller.&lt;/strong&gt; Not selected. The passage says she established a school, but neither the company nor the school survived her.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The passage does not tell whether it ceased to operate as a theater after Fuller died.&lt;/strong&gt; Not selected. This is a meta statement about missing information, not a positive fact about the theater at the Paris Exposition.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2682,7 @@
         <is>
           <t>Europe in the eleventh century underwent enormous social, technological, and economic changes, but this did not create a new Europe—it created two new ones. The north was developed as a rigidly hierarchical society in which status was determined, or was at least indicated, by the extent to which one owned, controlled, or labored on land; whereas the Mediterranean south developed a more fluid, and therefore more chaotic, world in which industry and commerce predominated and social status both reflected and resulted from the role that one played in the public life of the community. ln other words, individual identity and social community in the north were established on a personal basis, whereas in the south they were established on a civic basis. By the start of the twelfth century, northern and southern Europe were very different places indeed, and the Europeans themselves noticed it and commented on it.
 ---
-Which of the following was a deciding factor in person's place in society in northern and southern Europe respectively at the end of the eleventh century?
+Which of the following helped determine a person's place in society in northern or southern Europe at the end of the eleventh century?
 ---
 [] Ownership of a commercial enterprise.
 [] Participation in social and technological changes.
@@ -2956,49 +2692,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Understanding how to identify key information and distinguish between main ideas and supporting details is crucial for PTE Academic success. You're doing great by analyzing these passages!&lt;/p&gt;
-&lt;p&gt;The question asks us to identify the deciding factors for a person's social status in Northern and Southern Europe at the end of the eleventh century. The word "respectively" is important here, meaning the first factor would apply to the North and the second to the South, or that we are looking for factors that apply to *either* region as described.&lt;/p&gt;
-&lt;p&gt;Let's look at the passage again, focusing on how status was determined in each region:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Northern Europe:&lt;/strong&gt; "status was determined, or was at least indicated, by the extent to which one owned, controlled, or labored on land"&lt;/li&gt;
-    &lt;li&gt;&lt;strong&gt;Southern Europe:&lt;/strong&gt; "social status both reflected and resulted from the role that one played in the public life of the community."&lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Now, let's evaluate each option:&lt;/p&gt;
-&lt;h3&gt;Incorrect Options Explained:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Ownership of a commercial enterprise.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; While the passage mentions that in the Mediterranean south, "industry and commerce predominated," it does not explicitly state that the *ownership of a commercial enterprise* was the direct deciding factor for social status. Instead, it specifies that status in the South was determined by "the role that one played in the public life of the community." While owning a commercial enterprise might contribute to one's role in public life, it's not presented as the ultimate determinant of status itself. Furthermore, this factor is entirely irrelevant to Northern Europe, where land was the primary determinant.&lt;/li&gt;
-            &lt;li&gt;&lt;strong&gt;PTE Tip:&lt;/strong&gt; Be careful not to infer too much. Stick to what the passage explicitly states as the determining factor. "Predominated" means it was common or significant, but not necessarily the *deciding factor* for individual status.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Participation in social and technological changes.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; The passage states that "Europe in the eleventh century underwent enormous social, technological, and economic changes." This is a general statement about the era. However, the passage *does not* indicate that an individual's *participation* in these changes was a deciding factor for their social status in either Northern or Southern Europe. The passage clearly outlines specific determinants for status in each region (land in the North, public life in the South), neither of which is "participation in changes."&lt;/li&gt;
-            &lt;li&gt;&lt;strong&gt;PTE Tip:&lt;/strong&gt; Distinguish between background information or general context and the specific answers to the question. The passage describes the changes, but not how participating in them affected status.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Correct Options Explained:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Role in public life in the community.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; This option directly aligns with the description of Southern Europe. The passage explicitly states: "whereas the Mediterranean south developed a more fluid... world in which industry and commerce predominated and &lt;strong&gt;social status both reflected and resulted from the role that one played in the public life of the community&lt;/strong&gt;." This is a perfect match for the deciding factor in the South.&lt;/li&gt;
-            &lt;li&gt;&lt;strong&gt;PTE Tip:&lt;/strong&gt; Look for direct textual evidence. The phrasing in the option is almost identical to the passage's description of status in Southern Europe.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Relationship to land through ownership or labor.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; This option directly aligns with the description of Northern Europe. The passage states: "The north was developed as a rigidly hierarchical society in which &lt;strong&gt;status was determined, or was at least indicated, by the extent to which one owned, controlled, or labored on land&lt;/strong&gt;." This sentence clearly identifies the relationship to land (ownership or labor) as the deciding factor for social status in Northern Europe.&lt;/li&gt;
-            &lt;li&gt;&lt;strong&gt;PTE Tip:&lt;/strong&gt; Again, direct textual evidence is key. The passage explicitly links status in the North to land ownership, control, or labor.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;By carefully reading and identifying the specific details provided for each region, you can accurately determine the correct answers. Keep up the great work!&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Ownership of a commercial enterprise.&lt;/strong&gt; Not selected. The passage mentions industry and commerce in the south, but not commercial-enterprise ownership as the status marker.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Participation in social and technological changes.&lt;/strong&gt; Not selected. The passage describes changes in society, but does not say participation in those changes determined status.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Role in public life in the community.&lt;/strong&gt; Selected. For the Mediterranean south, the passage says social status resulted from the role one played in public life.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Relationship to land through ownership or labor.&lt;/strong&gt; Selected. For the north, the passage says status was determined or indicated by owning, controlling, or laboring on land.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -3493,50 +3187,16 @@
 ---
 Which of the following statements are true?
 ---
-[] Glucocorticoids work so bad for arthritis.
+[] Glucocorticoids work poorly for arthritis.
 [x] Aging can weaken our bones.
 [x] When we are young, there are fewer mineralocorticoid receptors in the bones than glucocorticoid receptors.
-[] Reducing the effect of glucocorticoid receptor must be a reasonable way to protect bone.
+[x] Reducing the impact of glucocorticoid receptors seemed like a logical way to protect bone.
 [x] Bone cells may be protected by drugs that block receptors.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Understanding how to identify correct and incorrect statements based on the passage is a crucial skill for the PTE Academic exam. We'll go through each option step-by-step.&lt;/p&gt;
-&lt;p&gt;Here's a detailed analysis of each statement:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Glucocorticoids work so bad for arthritis.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's Incorrect:&lt;/strong&gt; This statement directly contradicts the information provided in the passage. The third paragraph clearly states: "Drugs like prednisone are glucocorticoids, which are better known for their roles in reducing inflammation and suppressing the immune response, which is why they work &lt;strong&gt;so well&lt;/strong&gt; for problems like irritable bowel syndrome and arthritis." The passage indicates they are effective, not bad, for arthritis.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Aging can weaken our bones.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's Correct:&lt;/strong&gt; This statement is explicitly mentioned in the very first sentence of the passage: "Drugs we take can weaken our bones and &lt;strong&gt;so can aging&lt;/strong&gt;..." This makes it a straightforward true statement based on the text.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;When we are young, there are fewer mineralocorticoid receptors in the bones than glucocorticoid receptors.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's Correct:&lt;/strong&gt; Let's look at the fourth paragraph: "...bone, at least when we are young, has &lt;strong&gt;more glucocorticoid receptors than mineralocorticoid receptors&lt;/strong&gt;." If there are *more* glucocorticoid receptors, it logically follows that there are *fewer* mineralocorticoid receptors. This statement accurately rephrases the information given in the passage.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Reducing the effect of glucocorticoid receptor must be a reasonable way to protect bone.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's Incorrect:&lt;/strong&gt; While the last paragraph states, "So reducing the impact of glucocorticoid receptors &lt;strong&gt;seemed like a logical way&lt;/strong&gt; to protect bone," the word "must" in the option makes it too definitive and strong. The passage, particularly the first paragraph, hints that the "logical one" may not be the "best target." The scientists are finding that the mineralocorticoid receptor is a *key factor*, implying it might be a better or alternative target. The passage suggests it *seemed* logical, but doesn't confirm it *must* be the reasonable way, especially in light of new findings.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Bone cells may be protected by drugs that block receptors.&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's Correct:&lt;/strong&gt; The second paragraph clearly states: "And &lt;strong&gt;drugs that block the receptor&lt;/strong&gt;, like the hypertension medications spironolactone and eplerenone, &lt;strong&gt;may help protect bone cells&lt;/strong&gt;." This directly supports the statement, making it true.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! By carefully comparing each option to the exact wording and overall context of the passage, you can confidently identify the correct answers. Remember to pay close attention to qualifying words like "may," "must," "so well," or "seemed like" as they often hold the key to accuracy.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Glucocorticoids work poorly for arthritis.&lt;/strong&gt; Not selected. The passage says glucocorticoids work well for problems like arthritis.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Aging can weaken our bones.&lt;/strong&gt; Selected. The first sentence states that drugs can weaken bones and so can aging.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;When we are young, there are fewer mineralocorticoid receptors in the bones than glucocorticoid receptors.&lt;/strong&gt; Selected. The passage says young bone has more glucocorticoid receptors than mineralocorticoid receptors.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Reducing the impact of glucocorticoid receptors seemed like a logical way to protect bone.&lt;/strong&gt; Selected. The passage explicitly says reducing the impact of glucocorticoid receptors seemed like a logical way to protect bone.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Bone cells may be protected by drugs that block receptors.&lt;/strong&gt; Selected. The passage says drugs that block the mineralocorticoid receptor may help protect bone cells.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -3634,40 +3294,13 @@
 [] Increase collision damage.
 [x] Save the lives of pedestrians and drivers.
 [] Meet regulatory standards.
-[x] The normal operation.
+[x] Remain undamaged and operational after a high-impact crash.
 [x] Make our roads safer.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Understanding the nuances of language in passages is key to excelling in the PTE Academic test. We'll look at each option carefully and see how it relates to the information provided.&lt;/p&gt;
-&lt;h3&gt;Analysis of the Question and Passage:&lt;/h3&gt;
-&lt;p&gt;The question asks: &lt;strong&gt;"What are the functions of traffic lights that absorb kinetic energy?"&lt;/strong&gt; This means we need to identify the *purposes*, *roles*, or *outcomes* of this new technology as described in the passage.&lt;/p&gt;
-&lt;p&gt;The passage introduces a "game-changing technology" for traffic lights designed to "absorb kinetic energy, stopping them from crumpling when hit by a vehicle." It then details the benefits and goals of this innovation.&lt;/p&gt;
-&lt;h3&gt;Explanation of Options:&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Increase collision damage. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;This option is &lt;strong&gt;incorrect&lt;/strong&gt; because it directly contradicts the information in the passage. The text explicitly states that the project aims "to minimise collision-related injuries as well as damage to traffic lights and vehicles." The entire purpose of the technology is to *reduce* damage, not increase it.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Save the lives of pedestrians and drivers. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;This option is &lt;strong&gt;correct&lt;/strong&gt;. The passage clearly states that the technology "will prevent thousands of fatalities and injuries each year" and later, that it will "save pedestrian and motorists' lives." This is a primary function and benefit of the new traffic lights.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Meet regulatory standards. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;This option is &lt;strong&gt;incorrect&lt;/strong&gt;. While the passage mentions "while satisfying regulatory standards," this is a *design requirement* or a *condition* that the technology must meet, not a *function* it performs. The traffic lights don't *function* to meet standards; rather, they are *designed* to meet standards *while* performing their other functions (like regulating traffic, absorbing impact, and saving lives). The question asks for what the lights *do* or *achieve*, not the criteria they must fulfill to be implemented.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The normal operation. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;This option is &lt;strong&gt;correct&lt;/strong&gt;. The passage states that the goal is for the traffic lights to "remain undamaged and operational." "Operational" directly implies that they continue their normal function of regulating traffic, even after being hit. This is a significant benefit, as traditional lights might cease to function after an impact.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Make our roads safer. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;This option is &lt;strong&gt;correct&lt;/strong&gt;. The very first sentence of the passage states that this technology "will prevent thousands of fatalities and injuries each year and make our roads much safer." This is a direct and overarching function of the new traffic lights.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! By carefully distinguishing between functions, requirements, and contradictory information, you'll master these types of questions. You're doing well!&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Increase collision damage.&lt;/strong&gt; Not selected. The project aims to minimize injuries and damage, not increase collision damage.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Save the lives of pedestrians and drivers.&lt;/strong&gt; Selected. The passage says the technology can save pedestrian and motorists&amp;#x27; lives.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Meet regulatory standards.&lt;/strong&gt; Not selected. Satisfying regulatory standards is described as a design requirement, not a function of absorbing kinetic energy.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Remain undamaged and operational after a high-impact crash.&lt;/strong&gt; Selected. The passage says the lights should absorb a high-impact crash and remain undamaged and operational.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Make our roads safer.&lt;/strong&gt; Selected. The passage says the technology will prevent fatalities and injuries and make roads much safer.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -3694,46 +3327,12 @@
 [] Torrance Test of Creative Thinking can assess creativity.
 [x] The study lasted two years.
 [x] Torrance Test of Creative Thinking can solve real-world problems.
-[] Educating children in a way that encourages them to sympathize with others can improve their creativity.</t>
+[] Educating children in a way that encourages them to empathize with others can improve their creativity.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Your goal is to identify the statements that are **false** based on the provided passage. This requires careful reading and cross-referencing each option with the text.&lt;/p&gt;
-&lt;p&gt;Here’s a detailed analysis of each option:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The significant improvement of empathy promotes the overall creativity score. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect (i.e., why the statement is TRUE according to the passage):&lt;/strong&gt; The passage explicitly supports this statement. In the last paragraph, it says: "Pupils from the intervention school again scored much higher in these categories, indicating that a marked improvement in empathy was driving the overall creativity scores." This clearly states that improved empathy led to higher creativity scores. Since the statement is true, it is not one of the false statements we are looking for.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Torrance Test of Creative Thinking can assess creativity. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect (i.e., why the statement is TRUE according to the passage):&lt;/strong&gt; The third paragraph of the passage states: "Both sets of pupils were assessed for creativity at both the start and end of the school year using the Torrance Test of Creative Thinking: a well-established psychometric test." This sentence directly confirms that the Torrance Test is used to assess creativity. Since the statement is true, it is not one of the false statements.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The study lasted two years. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's correct (i.e., why the statement is FALSE according to the passage):&lt;/strong&gt; The second paragraph clearly states: "The findings are from a &lt;strong&gt;year-long&lt;/strong&gt; University of Cambridge study..." A "year-long" study means it lasted one year, not two. Therefore, this statement is false, making it a correct answer to the question.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Torrance Test of Creative Thinking can solve real-world problems. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's correct (i.e., why the statement is FALSE according to the passage):&lt;/strong&gt; The passage mentions "solving real-world problems" in the second paragraph, but it attributes this to the "engineering design thinking tools" used in the intervention group's D&amp;T lessons, not to the Torrance Test. The Torrance Test is described as a "psychometric test" used to "assess creativity." It is an assessment tool, not a problem-solving tool. Therefore, this statement is false, making it a correct answer.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Educating children in a way that encourages them to sympathize with others can improve their creativity. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;ul&gt;
-            &lt;li&gt;&lt;strong&gt;Why it's incorrect (i.e., why the statement is TRUE according to the passage):&lt;/strong&gt; The very first sentence of the passage states: "Teaching children in a way that encourages them to &lt;strong&gt;empathize&lt;/strong&gt; with others measurably improves their creativity..." While 'sympathize' and 'empathize' have subtle differences, in the context of encouraging understanding and connection with others to improve creativity, the passage's core finding supports this statement. The intervention aimed to "engender empathy" and led to improved creativity. Therefore, this statement is true according to the passage, and not one of the false statements.&lt;/li&gt;
-        &lt;/ul&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Identifying false statements requires precision and careful attention to detail, which you're clearly developing.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The question asks for statements that are false or incorrect, so selected answers are the statements that do not match the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;The significant improvement of empathy promotes the overall creativity score.&lt;/strong&gt; Not selected. This is true, so it is not selected for a false-statement question. The passage says improved empathy was driving the overall creativity scores.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Torrance Test of Creative Thinking can assess creativity.&lt;/strong&gt; Not selected. This is true, so it is not selected. The passage says pupils were assessed for creativity using the Torrance Test.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The study lasted two years.&lt;/strong&gt; Selected. This is false. The passage describes a year-long University of Cambridge study.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Torrance Test of Creative Thinking can solve real-world problems.&lt;/strong&gt; Selected. This is false. The engineering design thinking tools were used while solving real-world problems; the Torrance Test assessed creativity.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Educating children in a way that encourages them to empathize with others can improve their creativity.&lt;/strong&gt; Not selected. This is true, so it is not selected. The passage says teaching children to empathize measurably improves creativity.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -3929,8 +3528,8 @@
 ---
 According to the passage, which of the following statements about the Amazon protection is true?
 ---
-[x] The best way to protect the Amazon is to use laws governing human rights and probably international legislation.
-[] Protecting the rainforest is a vital top priority.
+[x] Using human rights law may be the best way to harness international legislation and tribunals to protect the Amazon.
+[x] Safeguarding the rainforest is a critical priority.
 [x] Using human rights law to protect the Amazon is more likely to prove promising.
 [x] The increase in regional deforestation and fires has made the protection more urgent.
 [] Protecting the Amazon is a common challenge of international law.</t>
@@ -3938,31 +3537,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. It's a fantastic way to sharpen your skills for the PTE Academic exam. We'll go through each option carefully, explaining why it's correct or incorrect based *only* on the information provided in the passage.&lt;/p&gt;
-&lt;p&gt;Here's a detailed analysis:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The best way to protect the Amazon is to use laws governing human rights and probably international legislation. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This statement is directly supported by the first sentence of the passage: "Using laws governing human rights &lt;strong&gt;may be the best way of harnessing international legislation and tribunals&lt;/strong&gt; to protect the Amazon..." The phrase "may be the best way" aligns perfectly with "the best way," and "harnessing international legislation" corresponds to "and probably international legislation." This option accurately reflects the main proposal of the study mentioned in the text.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Protecting the rainforest is a vital top priority. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage states, "Safeguarding the rainforest is a &lt;strong&gt;critical priority&lt;/strong&gt; because of the ecosystem's planetary importance." While "critical" and "vital" are very similar in meaning, the addition of "top" in the option makes it slightly different from what is explicitly stated. The passage says it's a "critical priority," implying it's extremely important, but it doesn't necessarily state it's *the* "top" or highest priority above all others. In PTE, it's crucial to stick as closely as possible to the exact wording and meaning presented in the text. "Critical priority" is strong, but "top priority" might be an overstatement or an inference not directly supported.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Using human rights law to protect the Amazon is more likely to prove promising. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This statement is directly supported by the third paragraph: "The new research... says using human rights law to protect the Amazon is &lt;strong&gt;more likely to have stronger prospects&lt;/strong&gt;..." The phrase "stronger prospects" is synonymous with "more likely to prove promising." This option accurately summarizes a key finding of the new study.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The increase in regional deforestation and fires has made the protection more urgent. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; This statement is explicitly mentioned in the second paragraph: "Recent increases in deforestation and fires in the region have made this &lt;strong&gt;even more urgent&lt;/strong&gt;." This is a direct match to the information in the passage.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Protecting the Amazon is a common challenge of international law. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Explanation:&lt;/strong&gt; The passage states, "The protection of the Amazon poses &lt;strong&gt;particular challenges&lt;/strong&gt; for international law..." The word "particular" means specific or unique, highlighting that these challenges are distinct to the Amazon's situation (e.g., due to territorial jurisdiction and sovereignty). "Common" implies widespread or frequently encountered, which is not what the passage suggests. The text emphasizes the *specific* difficulties, not that they are typical or common for international law in general.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Paying close attention to specific words and their nuances, as we did with "critical priority" versus "vital top priority," is a key skill for excelling in PTE reading. You're doing wonderfully!&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Using human rights law may be the best way to harness international legislation and tribunals to protect the Amazon.&lt;/strong&gt; Selected. The opening sentence states this directly.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Safeguarding the rainforest is a critical priority.&lt;/strong&gt; Selected. The passage states that safeguarding the rainforest is a critical priority because of its planetary importance.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Using human rights law to protect the Amazon is more likely to prove promising.&lt;/strong&gt; Selected. The passage says human rights law is more likely to have stronger prospects.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The increase in regional deforestation and fires has made the protection more urgent.&lt;/strong&gt; Selected. The passage states that recent increases in deforestation and fires have made protection even more urgent.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Protecting the Amazon is a common challenge of international law.&lt;/strong&gt; Not selected. The passage says Amazon protection poses particular challenges for international law, not common ones.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -4102,35 +3677,13 @@
 [x] Agrin can heal the wound instantly.
 [] Loss of ECM can delay wound healing.
 [] The expression of Agrin was enhanced when skin tissue was physically damaged.
-[] Chronic wound healing complications were the main reason for the decline of patients' emotional health.
+[] Chronic wound healing complications are a leading cause of decreased emotional well-being for patients.
 [x] One in 20 Singaporeans suffers from diabetes or burns.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. Your goal in PTE Academic is to carefully read the passage and determine which statements are truly supported or contradicted by the text. For this question, we're looking for the statements that are **incorrect** based on the information provided.&lt;/p&gt;
-&lt;p&gt;Here's a detailed analysis of each option:&lt;/p&gt;
-&lt;h3&gt;Agrin can heal the wound instantly. (Correct)&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why this statement is INCORRECT (and thus a 'Correct' answer to the question):&lt;/strong&gt; The passage states that Agrin has been discovered to "&lt;strong&gt;promote wound healing and repair&lt;/strong&gt;" and could "&lt;strong&gt;pave the way for the development of Agrin protein therapy to accelerate skin tissue healing&lt;/strong&gt;." The words "promote" and "accelerate" imply speeding up a process that still takes time, not an instantaneous cure. There is no mention of Agrin healing wounds instantly. Therefore, this statement is false according to the passage.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Loss of ECM can delay wound healing. (Incorrect)&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why this statement is CORRECT (and thus an 'Incorrect' answer to the question):&lt;/strong&gt; The passage explicitly states, "During injury, a major chunk of extracellular matrix, which helps to rebuild tissue, is lost, therefore &lt;strong&gt;delaying wound healing&lt;/strong&gt;." This directly supports the statement. Since the statement is true, it is not one of the "incorrect" statements we are looking for.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;The expression of Agrin was enhanced when skin tissue was physically damaged. (Incorrect)&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why this statement is CORRECT (and thus an 'Incorrect' answer to the question):&lt;/strong&gt; The passage clearly mentions, "Using both human and pre-clinical models, they found that physical injury to the skin tissue &lt;strong&gt;enhanced the expression of Agrin&lt;/strong&gt;..." This sentence directly confirms the statement. Since the statement is true, it is not one of the "incorrect" statements we are looking for.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;Chronic wound healing complications were the main reason for the decline of patients' emotional health. (Incorrect)&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why this statement is CORRECT (and thus an 'Incorrect' answer to the question):&lt;/strong&gt; The passage states that complications in chronic wound healing "are a &lt;strong&gt;leading cause&lt;/strong&gt; of amputation and &lt;strong&gt;decreased emotional well-being&lt;/strong&gt; for patients." While "leading cause" doesn't necessarily mean the *only* or *absolute main* reason, it strongly implies a primary and significant reason. In the context of the passage, it's presented as a major factor contributing to the decline in emotional health. Therefore, this statement is considered correct based on the passage's strong implication. Since the statement is true, it is not one of the "incorrect" statements we are looking for.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;h3&gt;One in 20 Singaporeans suffers from diabetes or burns. (Correct)&lt;/h3&gt;
-&lt;ul&gt;
-    &lt;li&gt;&lt;strong&gt;Why this statement is INCORRECT (and thus a 'Correct' answer to the question):&lt;/strong&gt; The passage states, "&lt;strong&gt;One in 20 Singaporeans is afflicted with chronic wound conditions&lt;/strong&gt;." It then clarifies that "Complications in the healing of chronic wounds are prevalent in patients suffering from diabetes or burn injuries." This means that diabetes and burns are *causes* of chronic wound conditions, but the statistic "One in 20" refers to the prevalence of *chronic wound conditions*, not specifically to the prevalence of diabetes or burns themselves. The statement incorrectly equates the statistic for chronic wounds with the prevalence of diabetes or burns. Therefore, this statement is false according to the passage.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Understanding these nuances is key to excelling in PTE Reading. You're doing well by carefully distinguishing between what the passage explicitly states and what it implies, versus what it does not mention or contradicts.&lt;/p&gt;</t>
+          <t>&lt;p&gt;The question asks for statements that are false or incorrect, so selected answers are the statements that do not match the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;Agrin can heal the wound instantly.&lt;/strong&gt; Selected. This is incorrect because the passage says Agrin may promote or accelerate healing, not heal wounds instantly.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Loss of ECM can delay wound healing.&lt;/strong&gt; Not selected. This statement is true: the passage says loss of extracellular matrix delays wound healing.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The expression of Agrin was enhanced when skin tissue was physically damaged.&lt;/strong&gt; Not selected. This statement is true: the passage says physical injury enhanced Agrin expression.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Chronic wound healing complications are a leading cause of decreased emotional well-being for patients.&lt;/strong&gt; Not selected. This statement is true: the passage describes chronic wound complications as a leading cause of decreased emotional well-being.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;One in 20 Singaporeans suffers from diabetes or burns.&lt;/strong&gt; Selected. This is incorrect because the one-in-20 statistic refers to chronic wound conditions, not diabetes or burns.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>
@@ -4217,42 +3770,14 @@
 [] What you eat has little to do with what you want to eat next.
 [] An unbalanced intake of macronutrients such as carbohydrates and protein is essential.
 [x] The fly senses macronutrients through its taste system.
-[] In the experiment, the researchers made sure the total calories in all three diets were the same.
+[x] In the experiment, the researchers made sure the total calories in all three diets were similar.
 [] The researchers tested the flies every two days for a week.
 [x] Dopamine in the brain is closely related to diet.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Hello there! Let's break down this reading comprehension question together. It's a great way to practice identifying key information and distinguishing between what the text explicitly states and what it doesn't. We'll go through each option step-by-step.&lt;/p&gt;
-&lt;p&gt;Here's a detailed explanation for each statement:&lt;/p&gt;
-&lt;ul&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;What you eat has little to do with what you want to eat next. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; This statement directly contradicts the very first sentence of the passage, which clearly states: "What you eat influences your taste for what you might want to eat next." The passage emphasizes a strong connection, not a weak one.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;An unbalanced intake of macronutrients such as carbohydrates and protein is essential. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; The passage states the exact opposite. It says, "Macronutrients like carbohydrates and proteins are essential; indeed, an unbalanced intake of these nutrients can be detrimental to health." So, an unbalanced intake is harmful ("detrimental"), not essential.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The fly senses macronutrients through its taste system. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; The passage explicitly supports this. It mentions, "Flies require macronutrients such as sugars and amino acids for survival. They use the gustatory system, the sensory system responsible for the perception of taste, to sense these nutrients and begin feeding." The "gustatory system" is defined as the "sensory system responsible for the perception of taste," confirming that flies use their taste system to sense macronutrients.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;In the experiment, the researchers made sure the total calories in all three diets were the same. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; This is a very subtle but important distinction in PTE. The passage states, "They ensured that all three diets were &lt;strong&gt;similar&lt;/strong&gt; in total calorie content..." While "similar" implies a close resemblance and an effort to control this variable, it does not necessarily mean they were "the same" (i.e., identical in calorie count). In scientific reporting, precision matters, and "similar" allows for slight variations, whereas "the same" implies exact equality. Therefore, stating they were "the same" is a stronger claim than what the passage supports.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;The researchers tested the flies every two days for a week. (Incorrect)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why it's incorrect:&lt;/strong&gt; The passage clearly states, "...and tested the flies &lt;strong&gt;daily&lt;/strong&gt; for a week to examine modifications in their food choice and taste sensitivity." "Daily" means every day, not every two days.&lt;/p&gt;
-    &lt;/li&gt;
-    &lt;li&gt;
-        &lt;p&gt;&lt;strong&gt;Dopamine in the brain is closely related to diet. (Correct)&lt;/strong&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Why it's correct:&lt;/strong&gt; The passage directly states, "The researchers report that diet affects dopamine and insulin signaling in the brain..." If diet "affects" dopamine signaling, it indicates a close relationship between the two. This effect then influences the flies' food choices, further solidifying the connection.&lt;/p&gt;
-    &lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Keep up the great work! Paying close attention to specific words and phrases in the passage, especially when comparing them to the options, is crucial for success in PTE reading tasks. You're doing well by analyzing each statement carefully!&lt;/p&gt;</t>
+          <t>&lt;p&gt;The selected answers are the statements directly supported by the passage.&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;strong&gt;What you eat has little to do with what you want to eat next.&lt;/strong&gt; Not selected. The passage says what you eat influences what you may want to eat next.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;An unbalanced intake of macronutrients such as carbohydrates and protein is essential.&lt;/strong&gt; Not selected. The passage says macronutrients are essential, but an unbalanced intake can be detrimental.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The fly senses macronutrients through its taste system.&lt;/strong&gt; Selected. The passage says flies use the gustatory system, the taste system, to sense these nutrients.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;In the experiment, the researchers made sure the total calories in all three diets were similar.&lt;/strong&gt; Selected. The passage says all three diets were similar in total calorie content.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;The researchers tested the flies every two days for a week.&lt;/strong&gt; Not selected. The passage says the flies were tested daily for a week.&lt;/li&gt;&lt;li&gt;&lt;strong&gt;Dopamine in the brain is closely related to diet.&lt;/strong&gt; Selected. The passage says diet affects dopamine and insulin signaling in the brain.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>